<commit_message>
Add updated output CSVs and code changes for signal filters
</commit_message>
<xml_diff>
--- a/data_ref/NSE_Stocks.xlsx
+++ b/data_ref/NSE_Stocks.xlsx
@@ -3786,7 +3786,7 @@
     <t>SMC GLOBAL SECURITIES LTD</t>
   </si>
   <si>
-    <t>NSE_EQ|INE337M01013</t>
+    <t>NSE_EQ|INE337M01021</t>
   </si>
   <si>
     <t>INDOTHAI</t>
@@ -8346,7 +8346,7 @@
     <t>RATEGAIN TRAVEL TECHN LTD</t>
   </si>
   <si>
-    <t>NSE_EQ|INE164B01022</t>
+    <t>NSE_EQ|INE164B01030</t>
   </si>
   <si>
     <t>KELLTONTEC</t>
@@ -18840,7 +18840,7 @@
       </c>
     </row>
     <row r="396" ht="15.75" customHeight="1">
-      <c r="A396" s="1" t="s">
+      <c r="A396" s="2" t="s">
         <v>1256</v>
       </c>
       <c r="B396" s="1" t="s">
@@ -27034,7 +27034,7 @@
       </c>
     </row>
     <row r="878" ht="15.75" customHeight="1">
-      <c r="A878" s="1" t="s">
+      <c r="A878" s="2" t="s">
         <v>2776</v>
       </c>
       <c r="B878" s="1" t="s">

</xml_diff>